<commit_message>
feat(phase3): add deposit short/over detector, platform fee vs net payout breakdown, and VAT invoice tracker
</commit_message>
<xml_diff>
--- a/docs/output/本月對帳差額與應收餘額表_202610.xlsx
+++ b/docs/output/本月對帳差額與應收餘額表_202610.xlsx
@@ -10,6 +10,7 @@
     <sheet name="對帳差額總表" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="玉山單筆沖銷對照" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="門市現金雙層審核與異常" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="平台手續費發票缺漏追蹤" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +584,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="19.5" customWidth="1" min="7" max="7"/>
-    <col width="51" customWidth="1" min="8" max="8"/>
+    <col width="67.5" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -645,7 +646,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>180718</v>
+        <v>186446</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>167270</v>
@@ -654,11 +655,11 @@
         <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>13448</v>
+        <v>19176</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>⏳ 門市尚有 $13,448 現金待存入銀行</t>
+          <t>⏳ 門市尚有 $19,176 現金待存入銀行</t>
         </is>
       </c>
     </row>
@@ -679,7 +680,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>254619</v>
+        <v>261117</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>228573</v>
@@ -688,11 +689,11 @@
         <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>26046</v>
+        <v>32544</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>⏳ 連加網路正常撥款作業中（約待撥 $26,046）</t>
+          <t>⏳ 連加網路撥款中（預估手續費 $752 / 實撥淨額 $31,792）</t>
         </is>
       </c>
     </row>
@@ -713,7 +714,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>50903</v>
+        <v>52523</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>28996</v>
@@ -722,11 +723,11 @@
         <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>21907</v>
+        <v>23527</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>⏳ Uber Eats 外送週期結算撥款中（約待撥 $21,907）</t>
+          <t>⏳ Uber Eats 結算中（預估抽成發票 $17,333 / 待撥淨額 $6,194）</t>
         </is>
       </c>
     </row>
@@ -747,7 +748,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1580</v>
+        <v>3970</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>1870</v>
@@ -756,11 +757,11 @@
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-290</v>
+        <v>2100</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>✅ 已全數結清沖銷</t>
+          <t>結算中（待撥 $2,100）</t>
         </is>
       </c>
     </row>
@@ -828,7 +829,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>⏳ 連加網路正常撥款作業中（約待撥 $75,090）</t>
+          <t>⏳ 連加網路撥款中（預估手續費 $1,735 / 實撥淨額 $73,355）</t>
         </is>
       </c>
     </row>
@@ -862,7 +863,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>⏳ Uber Eats 外送週期結算撥款中（約待撥 $11,032）</t>
+          <t>⏳ Uber Eats 結算中（預估抽成發票 $5,390 / 待撥淨額 $5,642）</t>
         </is>
       </c>
     </row>
@@ -896,7 +897,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>⏳ Foodpanda 外送週期結算撥款中（約待撥 $15,596）</t>
+          <t>⏳ Foodpanda 結算中（預估抽成發票 $5,240 / 待撥淨額 $10,356）</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3270,10 +3271,11 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="79.5" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22.5" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="106.5" customWidth="1" min="9" max="9"/>
+    <col width="40.5" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="22.5" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="157.5" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3304,20 +3306,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>短溢差額 (實存-應收)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>第二層：玉山銀行入帳狀態</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>雙層審核結論</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>已延遲天數</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>處置建議</t>
         </is>
@@ -3347,20 +3354,25 @@
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G2" s="19" t="inlineStr">
+      <c r="H2" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>8 天</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/16 存入 $31,720 (2026-10-14~2026-10-15累計))</t>
         </is>
@@ -3390,20 +3402,25 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G3" s="19" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>7 天</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/16 存入 $31,720 (2026-10-14~2026-10-15累計))</t>
         </is>
@@ -3433,20 +3450,25 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="H4" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>6 天</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/19 存入 $44,659 (2026-10-16~2026-10-18累計))</t>
         </is>
@@ -3476,20 +3498,25 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G5" s="19" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>5 天</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/19 存入 $44,659 (2026-10-16~2026-10-18累計))</t>
         </is>
@@ -3519,20 +3546,25 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="H6" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>4 天</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/19 存入 $44,659 (2026-10-16~2026-10-18累計))</t>
         </is>
@@ -3562,22 +3594,27 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
+          <t>⚠️ 短少 -$1,020 (應收合 $25,990)</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>3 天</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/21 存入 $24,970 (2026-10-19~2026-10-20累計))</t>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>【注意短溢：⚠️ 短少 -$1,020 (應收合 $25,990)】總表已登記提存，待存摺更新自動結清 (申報於 2026/10/21 存入 $24,970 (2026-10-19~2026-10-20累計))</t>
         </is>
       </c>
     </row>
@@ -3605,20 +3642,25 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
+          <t>⏳ 待存入</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
           <t>❌ 存摺未見入帳</t>
         </is>
       </c>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>🔴 門市未存 (留店未存)</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>2 天</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>門市正常交班處理中，待總表申報或存款</t>
         </is>
@@ -3648,22 +3690,27 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
+          <t>⚠️ 短少 -$1,020 (應收合 $25,990)</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
           <t>⏳ 存摺尚未到帳/未更新</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="H9" s="19" t="inlineStr">
         <is>
           <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>2 天</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/21 存入 $24,970 (2026-10-19~2026-10-20累計))</t>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>【注意短溢：⚠️ 短少 -$1,020 (應收合 $25,990)】總表已登記提存，待存摺更新自動結清 (申報於 2026/10/21 存入 $24,970 (2026-10-19~2026-10-20累計))</t>
         </is>
       </c>
     </row>
@@ -3691,20 +3738,25 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
+          <t>⏳ 待存入</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
           <t>❌ 存摺未見入帳</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>🔴 門市未存 (留店未存)</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>1 天</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>門市正常交班處理中，待總表申報或存款</t>
         </is>
@@ -3734,22 +3786,373 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
+          <t>⏳ 待存入</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
           <t>❌ 存摺未見入帳</t>
         </is>
       </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="H11" s="20" t="inlineStr">
         <is>
           <t>🔴 門市未存 (留店未存)</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="I11" s="10" t="inlineStr">
         <is>
           <t>1 天</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>門市正常交班處理中，待總表申報或存款</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>月宮 (月下餐飲)</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>5728</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>❌ 總表U欄空白未填</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 待存入</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>❌ 存摺未見入帳</t>
+        </is>
+      </c>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>🔴 門市未存 (留店未存)</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>0 天</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>門市正常交班處理中，待總表申報或存款</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16.5" customWidth="1" min="6" max="6"/>
+    <col width="19.5" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22.5" customWidth="1" min="9" max="9"/>
+    <col width="75" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>事業體</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>平台名稱</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>廠商統編</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>抽成/手續費率</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>本月 POS 營收</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>預估全月手續費含稅總額</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>預估可扣抵 5% 進項稅額</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>已匯入發票沖銷</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>目前發票追蹤狀態</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>會計核對與索取建議</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>月宮 (月下餐飲)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LINE Pay (連加網路)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>99024139</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2.31%</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="n">
+        <v>261117</v>
+      </c>
+      <c r="F2" s="12" t="n">
+        <v>3319</v>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>🟡 傳票已提列・待核對月底發票</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>月底核對連加網路 (99024139) 電子發票約 $3,319（含可扣抵進項稅額 $158）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>月宮 (月下餐飲)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Uber Eats (優步科技)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>83118125</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>約 33%</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>52523</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>17333</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>825</v>
+      </c>
+      <c r="H3" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>🔴 待取得發票沖銷差額</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>請下載優步 (83118125) 手續費發票約 $17,333 沖銷應收差額（可扣抵稅額 $825）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LINE Pay (連加網路)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>99024139</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2.31%</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>170122</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>2777</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>132</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>🟡 傳票已提列・待核對月底發票</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>月底核對連加網路 (99024139) 電子發票約 $2,777（含可扣抵進項稅額 $132）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Uber Eats (優步科技)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>83118125</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>約 33%</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>16333</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>5390</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>257</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>🔴 待取得發票沖銷差額</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>請下載優步 (83118125) 手續費發票約 $5,390 沖銷應收差額（可扣抵稅額 $257）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Foodpanda (富胖達)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>53075607</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>約 33.6%</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>15596</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>5240</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>🔴 待取得發票沖銷差額</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>請下載富胖達 (53075607) 手續費發票約 $5,240 沖銷應收差額（可扣抵稅額 $250）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(invoice): add invoice upload & registration modal with real-time fee deduction and VAT calculation
</commit_message>
<xml_diff>
--- a/docs/output/本月對帳差額與應收餘額表_202610.xlsx
+++ b/docs/output/本月對帳差額與應收餘額表_202610.xlsx
@@ -3929,7 +3929,7 @@
     <col width="19.5" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="22.5" customWidth="1" min="9" max="9"/>
-    <col width="75" customWidth="1" min="10" max="10"/>
+    <col width="64.5" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>月底核對連加網路 (99024139) 電子發票約 $6,042（含可扣抵進項稅額 $288）</t>
+          <t>連加網路 (99024139) 手續費約 $6,042（含可扣抵進項稅額 $288）</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>請下載優步 (83118125) 手續費發票約 $17,333 沖銷應收差額（可扣抵稅額 $825）</t>
+          <t>優步科技 (83118125) 手續費發票約 $17,333（含可扣抵稅額 $825）</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>月底核對連加網路 (99024139) 電子發票約 $4,075（含可扣抵進項稅額 $194）</t>
+          <t>連加網路 (99024139) 手續費約 $4,075（含可扣抵進項稅額 $194）</t>
         </is>
       </c>
     </row>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>請下載優步 (83118125) 手續費發票約 $5,068 沖銷應收差額（可扣抵稅額 $241）</t>
+          <t>優步科技 (83118125) 手續費發票約 $5,068（含可扣抵稅額 $241）</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>請下載富胖達 (53075607) 手續費發票約 $5,352 沖銷應收差額（可扣抵稅額 $255）</t>
+          <t>富胖達 (53075607) 手續費發票約 $5,352（含可扣抵稅額 $255）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reconcile): update reconciliation snapshot at 2026-10-30 11:32:16
</commit_message>
<xml_diff>
--- a/docs/output/本月對帳差額與應收餘額表_202610.xlsx
+++ b/docs/output/本月對帳差額與應收餘額表_202610.xlsx
@@ -646,20 +646,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>209565</v>
+        <v>230206</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>209565</v>
+        <v>230206</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>191786</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>17779</v>
+        <v>38420</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收現金 $209,565 / 已存現金 $191,786 ➔ 待入帳 $17,779</t>
+          <t>⏳ 實收現金 $230,206 / 已存現金 $191,786 ➔ 待入帳 $38,420</t>
         </is>
       </c>
     </row>
@@ -680,20 +680,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>303640</v>
+        <v>320710</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>296613</v>
+        <v>313212</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>261323</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>35290</v>
+        <v>51889</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收LINE Pay $296,613 / 已存 $261,323 ➔ 待入帳 $35,290</t>
+          <t>⏳ 實收LINE Pay $313,212 / 已存 $261,323 ➔ 待入帳 $51,889</t>
         </is>
       </c>
     </row>
@@ -714,20 +714,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>64003</v>
+        <v>67408</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>42882</v>
+        <v>45163</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>28996</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>13886</v>
+        <v>16167</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收Uber Eats $42,882 / 已存 $28,996 ➔ 待入帳 $13,886</t>
+          <t>⏳ 實收Uber Eats $45,163 / 已存 $28,996 ➔ 待入帳 $16,167</t>
         </is>
       </c>
     </row>
@@ -782,20 +782,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>384727</v>
+        <v>424705</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>384727</v>
+        <v>424705</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>209228</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>175499</v>
+        <v>215477</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收現金 $384,727 / 已存現金 $209,228 ➔ 待入帳 $175,499</t>
+          <t>⏳ 實收現金 $424,705 / 已存現金 $209,228 ➔ 待入帳 $215,477</t>
         </is>
       </c>
     </row>
@@ -816,20 +816,20 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>194432</v>
+        <v>215240</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>189933</v>
+        <v>210260</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>93990</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>95943</v>
+        <v>116270</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收LINE Pay $189,933 / 已存 $93,990 ➔ 待入帳 $95,943</t>
+          <t>⏳ 實收LINE Pay $210,260 / 已存 $93,990 ➔ 待入帳 $116,270</t>
         </is>
       </c>
     </row>
@@ -850,20 +850,20 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>20140</v>
+        <v>20787</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>13890</v>
+        <v>14336</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>5301</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>8589</v>
+        <v>9035</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收Uber Eats $13,890 / 已存 $5,301 ➔ 待入帳 $8,589</t>
+          <t>⏳ 實收Uber Eats $14,336 / 已存 $5,301 ➔ 待入帳 $9,035</t>
         </is>
       </c>
     </row>
@@ -884,20 +884,20 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>19080</v>
+        <v>21286</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>12669</v>
+        <v>14134</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>12669</v>
+        <v>14134</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>⏳ 實收Foodpanda $12,669 / 已存 $0 ➔ 待入帳 $12,669</t>
+          <t>⏳ 實收Foodpanda $14,134 / 已存 $0 ➔ 待入帳 $14,134</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4139,22 +4139,22 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>❌ 總表U欄空白未填</t>
+          <t>✅ 申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計)</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>⏳ 待存入</t>
+          <t>✓ 金額相符</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>❌ 存摺未見入帳</t>
-        </is>
-      </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>🔴 門市未存 (留店未存)</t>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>門市正常交班處理中，待總表申報或存款</t>
+          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計))</t>
         </is>
       </c>
     </row>
@@ -4187,22 +4187,22 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>❌ 總表U欄空白未填</t>
+          <t>✅ 申報於 2026/10/27 存入 $25,361 (2026-10-26~2026-10-28累計)</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>⏳ 待存入</t>
+          <t>➕ 溢存 +$780 (應收合 $24,581)</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>❌ 存摺未見入帳</t>
-        </is>
-      </c>
-      <c r="H11" s="20" t="inlineStr">
-        <is>
-          <t>🔴 門市未存 (留店未存)</t>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>門市正常交班處理中，待總表申報或存款</t>
+          <t>【注意短溢：➕ 溢存 +$780 (應收合 $24,581)】總表已登記提存，待存摺更新自動結清 (申報於 2026/10/27 存入 $25,361 (2026-10-26~2026-10-28累計))</t>
         </is>
       </c>
     </row>
@@ -4235,22 +4235,22 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>❌ 總表U欄空白未填</t>
+          <t>✅ 申報於 2026/10/27 存入 $25,361 (2026-10-26~2026-10-28累計)</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>⏳ 待存入</t>
+          <t>➕ 溢存 +$780 (應收合 $24,581)</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>❌ 存摺未見入帳</t>
-        </is>
-      </c>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>🔴 門市未存 (留店未存)</t>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>門市正常交班處理中，待總表申報或存款</t>
+          <t>【注意短溢：➕ 溢存 +$780 (應收合 $24,581)】總表已登記提存，待存摺更新自動結清 (申報於 2026/10/27 存入 $25,361 (2026-10-26~2026-10-28累計))</t>
         </is>
       </c>
     </row>
@@ -4270,35 +4270,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>隨意小吃</t>
+          <t>月宮 (月下餐飲)</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13890</v>
+        <v>13273</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>❌ 總表U欄空白未填</t>
+          <t>✅ 申報於 2026/10/27 存入 $25,361 (2026-10-26~2026-10-28累計)</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>⏳ 待存入</t>
+          <t>➕ 溢存 +$780 (應收合 $24,581)</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>❌ 存摺未見入帳</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t>🔴 門市未存 (留店未存)</t>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>門市正常交班處理中，待總表申報或存款</t>
+          <t>【注意短溢：➕ 溢存 +$780 (應收合 $24,581)】總表已登記提存，待存摺更新自動結清 (申報於 2026/10/27 存入 $25,361 (2026-10-26~2026-10-28累計))</t>
         </is>
       </c>
     </row>
@@ -4318,16 +4318,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>隨意小吃</t>
+          <t>月宮 (月下餐飲)</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="D14" s="12" t="n">
-        <v>18100</v>
+        <v>7368</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -4371,30 +4371,30 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>14830</v>
+        <v>13890</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>❌ 總表U欄空白未填</t>
+          <t>✅ 申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>⏳ 待存入</t>
+          <t>✓ 金額相符</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>❌ 存摺未見入帳</t>
-        </is>
-      </c>
-      <c r="H15" s="20" t="inlineStr">
-        <is>
-          <t>🔴 門市未存 (留店未存)</t>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>門市正常交班處理中，待總表申報或存款</t>
+          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計))</t>
         </is>
       </c>
     </row>
@@ -4419,38 +4419,230 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>18100</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>✅ 申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計)</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>0 天</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計))</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>14830</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>✅ 申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計)</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>0 天</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計))</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D18" s="12" t="n">
         <v>15490</v>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>✅ 申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計)</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>✓ 金額相符</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 存摺尚未到帳/未更新</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>🟡 門市已申報 (待銀行入帳)</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>0 天</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>總表已登記提存，待存摺更新自動結清 (申報於 2026/10/28 存入 $73,130 (2026-10-21~2026-10-27累計))</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>19380</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>❌ 總表U欄空白未填</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>⏳ 待存入</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>❌ 存摺未見入帳</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H19" s="20" t="inlineStr">
         <is>
           <t>🔴 門市未存 (留店未存)</t>
         </is>
       </c>
-      <c r="I16" s="10" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>0 天</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>門市正常交班處理中，待總表申報或存款</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>隨意小吃</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>20598</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>❌ 總表U欄空白未填</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 待存入</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>❌ 存摺未見入帳</t>
+        </is>
+      </c>
+      <c r="H20" s="20" t="inlineStr">
+        <is>
+          <t>🔴 門市未存 (留店未存)</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>0 天</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>門市正常交班處理中，待總表申報或存款</t>
         </is>
@@ -4556,13 +4748,13 @@
         </is>
       </c>
       <c r="E2" s="12" t="n">
-        <v>303640</v>
+        <v>320710</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>7027</v>
+        <v>7498</v>
       </c>
       <c r="G2" s="12" t="n">
-        <v>335</v>
+        <v>357</v>
       </c>
       <c r="H2" s="12" t="n">
         <v>0</v>
@@ -4574,7 +4766,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>連加網路 (99024139) 手續費約 $7,027（含可扣抵進項稅額 $335）</t>
+          <t>連加網路 (99024139) 手續費約 $7,498（含可扣抵進項稅額 $357）</t>
         </is>
       </c>
     </row>
@@ -4600,13 +4792,13 @@
         </is>
       </c>
       <c r="E3" s="12" t="n">
-        <v>64003</v>
+        <v>67408</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>21121</v>
+        <v>22245</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>1006</v>
+        <v>1059</v>
       </c>
       <c r="H3" s="12" t="n">
         <v>0</v>
@@ -4618,7 +4810,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>優步科技 (83118125) 手續費發票約 $21,121（含可扣抵稅額 $1,006）</t>
+          <t>優步科技 (83118125) 手續費發票約 $22,245（含可扣抵稅額 $1,059）</t>
         </is>
       </c>
     </row>
@@ -4644,13 +4836,13 @@
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>194432</v>
+        <v>215240</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>4499</v>
+        <v>4980</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>214</v>
+        <v>237</v>
       </c>
       <c r="H4" s="12" t="n">
         <v>0</v>
@@ -4662,7 +4854,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>連加網路 (99024139) 手續費約 $4,499（含可扣抵進項稅額 $214）</t>
+          <t>連加網路 (99024139) 手續費約 $4,980（含可扣抵進項稅額 $237）</t>
         </is>
       </c>
     </row>
@@ -4688,13 +4880,13 @@
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>20140</v>
+        <v>20787</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6250</v>
+        <v>6451</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="H5" s="12" t="n">
         <v>0</v>
@@ -4706,7 +4898,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>優步科技 (83118125) 手續費發票約 $6,250（含可扣抵稅額 $298）</t>
+          <t>優步科技 (83118125) 手續費發票約 $6,451（含可扣抵稅額 $307）</t>
         </is>
       </c>
     </row>
@@ -4732,13 +4924,13 @@
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>19080</v>
+        <v>21286</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>6411</v>
+        <v>7152</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>305</v>
+        <v>341</v>
       </c>
       <c r="H6" s="12" t="n">
         <v>0</v>
@@ -4750,7 +4942,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>富胖達 (53075607) 手續費發票約 $6,411（含可扣抵稅額 $305）</t>
+          <t>富胖達 (53075607) 手續費發票約 $7,152（含可扣抵稅額 $341）</t>
         </is>
       </c>
     </row>

</xml_diff>